<commit_message>
put clustered sentences and yaml files
</commit_message>
<xml_diff>
--- a/clustered_sentences.xlsx
+++ b/clustered_sentences.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gx1/Git/Unina/peac-experiment/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{C892F763-C227-B245-8E08-E3876C4E418C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{EF80FF1F-3C4C-D043-AF69-973F10E68100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5540" yWindow="2300" windowWidth="27700" windowHeight="16940" xr2:uid="{A56C1C2B-3A0B-304A-84FE-95D49B9BBDCF}"/>
+    <workbookView xWindow="2540" yWindow="1480" windowWidth="27700" windowHeight="16940" xr2:uid="{A56C1C2B-3A0B-304A-84FE-95D49B9BBDCF}"/>
   </bookViews>
   <sheets>
     <sheet name="clustered_sentences" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="12766" uniqueCount="3113">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="12798" uniqueCount="3121">
   <si>
     <t>cluster_id</t>
   </si>
@@ -9387,6 +9387,30 @@
   </si>
   <si>
     <t>examples/analogy.yaml</t>
+  </si>
+  <si>
+    <t>examples/visual_resonance.yaml</t>
+  </si>
+  <si>
+    <t>format/skincare.yaml</t>
+  </si>
+  <si>
+    <t>tone/storyteller.yaml</t>
+  </si>
+  <si>
+    <t>markdown/markdown.yaml, markdown/bullet.yaml</t>
+  </si>
+  <si>
+    <t>tone/resilient.yaml</t>
+  </si>
+  <si>
+    <t>format/same.yaml</t>
+  </si>
+  <si>
+    <t>format/same.yaml,format/more_literary.yaml</t>
+  </si>
+  <si>
+    <t>examples/stories.yaml</t>
   </si>
 </sst>
 </file>
@@ -11580,6 +11604,9 @@
       <c r="D82" s="2" t="s">
         <v>2716</v>
       </c>
+      <c r="E82" s="1" t="s">
+        <v>3113</v>
+      </c>
     </row>
     <row r="83" spans="1:6" ht="20" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
@@ -11594,6 +11621,9 @@
       <c r="D83" s="2" t="s">
         <v>2720</v>
       </c>
+      <c r="E83" s="1" t="s">
+        <v>3113</v>
+      </c>
     </row>
     <row r="84" spans="1:6" ht="40" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
@@ -11608,6 +11638,9 @@
       <c r="D84" s="2" t="s">
         <v>2709</v>
       </c>
+      <c r="E84" s="1" t="s">
+        <v>3113</v>
+      </c>
     </row>
     <row r="85" spans="1:6" ht="40" x14ac:dyDescent="0.25">
       <c r="A85" s="1">
@@ -11792,7 +11825,7 @@
         <v>2396</v>
       </c>
     </row>
-    <row r="97" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A97" s="1">
         <v>25</v>
       </c>
@@ -11806,7 +11839,7 @@
         <v>1818</v>
       </c>
     </row>
-    <row r="98" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A98" s="1">
         <v>25</v>
       </c>
@@ -11820,7 +11853,7 @@
         <v>1834</v>
       </c>
     </row>
-    <row r="99" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
         <v>26</v>
       </c>
@@ -11834,7 +11867,7 @@
         <v>1028</v>
       </c>
     </row>
-    <row r="100" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A100" s="1">
         <v>26</v>
       </c>
@@ -11848,7 +11881,7 @@
         <v>1023</v>
       </c>
     </row>
-    <row r="101" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A101" s="1">
         <v>27</v>
       </c>
@@ -11862,7 +11895,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="102" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A102" s="1">
         <v>27</v>
       </c>
@@ -11876,7 +11909,7 @@
         <v>1380</v>
       </c>
     </row>
-    <row r="103" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A103" s="1">
         <v>28</v>
       </c>
@@ -11889,8 +11922,11 @@
       <c r="D103" s="2" t="s">
         <v>2928</v>
       </c>
-    </row>
-    <row r="104" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+      <c r="E103" s="1" t="s">
+        <v>3114</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A104" s="1">
         <v>28</v>
       </c>
@@ -11903,8 +11939,11 @@
       <c r="D104" s="2" t="s">
         <v>2924</v>
       </c>
-    </row>
-    <row r="105" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+      <c r="E104" s="1" t="s">
+        <v>3114</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A105" s="1">
         <v>29</v>
       </c>
@@ -11918,7 +11957,7 @@
         <v>1821</v>
       </c>
     </row>
-    <row r="106" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A106" s="1">
         <v>29</v>
       </c>
@@ -11932,7 +11971,7 @@
         <v>1832</v>
       </c>
     </row>
-    <row r="107" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A107" s="1">
         <v>30</v>
       </c>
@@ -11946,7 +11985,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="108" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A108" s="1">
         <v>30</v>
       </c>
@@ -11960,7 +11999,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="109" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A109" s="1">
         <v>30</v>
       </c>
@@ -11974,7 +12013,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="110" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A110" s="1">
         <v>31</v>
       </c>
@@ -11988,7 +12027,7 @@
         <v>1817</v>
       </c>
     </row>
-    <row r="111" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A111" s="1">
         <v>31</v>
       </c>
@@ -12002,7 +12041,7 @@
         <v>631</v>
       </c>
     </row>
-    <row r="112" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A112" s="1">
         <v>32</v>
       </c>
@@ -12192,6 +12231,9 @@
       <c r="D124" s="2" t="s">
         <v>2506</v>
       </c>
+      <c r="E124" s="1" t="s">
+        <v>3115</v>
+      </c>
     </row>
     <row r="125" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A125" s="1">
@@ -12206,6 +12248,9 @@
       <c r="D125" s="2" t="s">
         <v>2104</v>
       </c>
+      <c r="E125" s="1" t="s">
+        <v>3115</v>
+      </c>
     </row>
     <row r="126" spans="1:5" ht="20" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="1">
@@ -12237,6 +12282,9 @@
       <c r="D127" s="2" t="s">
         <v>2736</v>
       </c>
+      <c r="E127" s="1" t="s">
+        <v>3115</v>
+      </c>
     </row>
     <row r="128" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A128" s="1">
@@ -12251,6 +12299,9 @@
       <c r="D128" s="2" t="s">
         <v>2101</v>
       </c>
+      <c r="E128" s="1" t="s">
+        <v>3115</v>
+      </c>
     </row>
     <row r="129" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A129" s="1">
@@ -15340,6 +15391,9 @@
       <c r="D312" s="2" t="s">
         <v>364</v>
       </c>
+      <c r="E312" s="1" t="s">
+        <v>3075</v>
+      </c>
     </row>
     <row r="313" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A313" s="1">
@@ -15354,6 +15408,9 @@
       <c r="D313" s="2" t="s">
         <v>456</v>
       </c>
+      <c r="E313" s="1" t="s">
+        <v>3116</v>
+      </c>
     </row>
     <row r="314" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A314" s="1">
@@ -15687,6 +15744,9 @@
       <c r="D334" s="2" t="s">
         <v>2025</v>
       </c>
+      <c r="E334" s="1" t="s">
+        <v>3111</v>
+      </c>
       <c r="F334" s="1" t="s">
         <v>3105</v>
       </c>
@@ -15738,6 +15798,9 @@
       <c r="D337" s="2" t="s">
         <v>1860</v>
       </c>
+      <c r="E337" s="1" t="s">
+        <v>3081</v>
+      </c>
       <c r="F337" s="1" t="s">
         <v>3105</v>
       </c>
@@ -15772,6 +15835,9 @@
       <c r="D339" s="2" t="s">
         <v>2214</v>
       </c>
+      <c r="E339" s="1" t="s">
+        <v>3083</v>
+      </c>
     </row>
     <row r="340" spans="1:6" ht="40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A340" s="1">
@@ -16092,6 +16158,9 @@
       <c r="D358" s="2" t="s">
         <v>500</v>
       </c>
+      <c r="E358" s="1" t="s">
+        <v>3083</v>
+      </c>
     </row>
     <row r="359" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A359" s="1">
@@ -16106,6 +16175,9 @@
       <c r="D359" s="2" t="s">
         <v>715</v>
       </c>
+      <c r="E359" s="1" t="s">
+        <v>3117</v>
+      </c>
     </row>
     <row r="360" spans="1:5" ht="40" hidden="1" x14ac:dyDescent="0.25">
       <c r="A360" s="1">
@@ -16137,6 +16209,9 @@
       <c r="D361" s="2" t="s">
         <v>1679</v>
       </c>
+      <c r="E361" s="1" t="s">
+        <v>3117</v>
+      </c>
     </row>
     <row r="362" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A362" s="1">
@@ -16179,6 +16254,9 @@
       <c r="D364" s="2" t="s">
         <v>2001</v>
       </c>
+      <c r="E364" s="1" t="s">
+        <v>3083</v>
+      </c>
     </row>
     <row r="365" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A365" s="1">
@@ -16193,6 +16271,9 @@
       <c r="D365" s="2" t="s">
         <v>563</v>
       </c>
+      <c r="E365" s="1" t="s">
+        <v>3083</v>
+      </c>
     </row>
     <row r="366" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A366" s="1">
@@ -16207,6 +16288,9 @@
       <c r="D366" s="2" t="s">
         <v>236</v>
       </c>
+      <c r="E366" s="1" t="s">
+        <v>3083</v>
+      </c>
     </row>
     <row r="367" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A367" s="1">
@@ -16239,7 +16323,7 @@
         <v>3057</v>
       </c>
     </row>
-    <row r="369" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A369" s="1">
         <v>68</v>
       </c>
@@ -16252,8 +16336,11 @@
       <c r="D369" s="2" t="s">
         <v>1261</v>
       </c>
-    </row>
-    <row r="370" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+      <c r="E369" s="1" t="s">
+        <v>3118</v>
+      </c>
+    </row>
+    <row r="370" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A370" s="1">
         <v>68</v>
       </c>
@@ -16266,8 +16353,11 @@
       <c r="D370" s="2" t="s">
         <v>794</v>
       </c>
-    </row>
-    <row r="371" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+      <c r="E370" s="1" t="s">
+        <v>3119</v>
+      </c>
+    </row>
+    <row r="371" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A371" s="1">
         <v>69</v>
       </c>
@@ -16281,7 +16371,7 @@
         <v>2337</v>
       </c>
     </row>
-    <row r="372" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A372" s="1">
         <v>69</v>
       </c>
@@ -16294,8 +16384,11 @@
       <c r="D372" s="2" t="s">
         <v>2327</v>
       </c>
-    </row>
-    <row r="373" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+      <c r="E372" s="1" t="s">
+        <v>3057</v>
+      </c>
+    </row>
+    <row r="373" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A373" s="1">
         <v>69</v>
       </c>
@@ -16308,8 +16401,11 @@
       <c r="D373" s="2" t="s">
         <v>2592</v>
       </c>
-    </row>
-    <row r="374" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="E373" s="1" t="s">
+        <v>3057</v>
+      </c>
+    </row>
+    <row r="374" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A374" s="1">
         <v>72</v>
       </c>
@@ -16323,7 +16419,7 @@
         <v>2241</v>
       </c>
     </row>
-    <row r="375" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A375" s="1">
         <v>72</v>
       </c>
@@ -16337,7 +16433,7 @@
         <v>2235</v>
       </c>
     </row>
-    <row r="376" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A376" s="1">
         <v>72</v>
       </c>
@@ -16351,7 +16447,7 @@
         <v>2231</v>
       </c>
     </row>
-    <row r="377" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A377" s="1">
         <v>74</v>
       </c>
@@ -16365,7 +16461,7 @@
         <v>1773</v>
       </c>
     </row>
-    <row r="378" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A378" s="1">
         <v>74</v>
       </c>
@@ -16379,7 +16475,7 @@
         <v>1771</v>
       </c>
     </row>
-    <row r="379" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A379" s="1">
         <v>75</v>
       </c>
@@ -16393,7 +16489,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="380" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A380" s="1">
         <v>75</v>
       </c>
@@ -16407,7 +16503,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="381" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A381" s="1">
         <v>76</v>
       </c>
@@ -16421,7 +16517,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="382" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A382" s="1">
         <v>76</v>
       </c>
@@ -16435,7 +16531,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="383" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A383" s="1">
         <v>77</v>
       </c>
@@ -16449,7 +16545,7 @@
         <v>2623</v>
       </c>
     </row>
-    <row r="384" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A384" s="1">
         <v>78</v>
       </c>
@@ -16490,6 +16586,9 @@
       <c r="D386" s="2" t="s">
         <v>2350</v>
       </c>
+      <c r="E386" s="1" t="s">
+        <v>3083</v>
+      </c>
     </row>
     <row r="387" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A387" s="1">
@@ -16504,6 +16603,9 @@
       <c r="D387" s="2" t="s">
         <v>1645</v>
       </c>
+      <c r="E387" s="1" t="s">
+        <v>3083</v>
+      </c>
     </row>
     <row r="388" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A388" s="1">
@@ -16682,6 +16784,9 @@
       <c r="D398" s="2" t="s">
         <v>2551</v>
       </c>
+      <c r="E398" s="1" t="s">
+        <v>3080</v>
+      </c>
     </row>
     <row r="399" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A399" s="1">
@@ -16696,6 +16801,9 @@
       <c r="D399" s="2" t="s">
         <v>759</v>
       </c>
+      <c r="E399" s="1" t="s">
+        <v>3080</v>
+      </c>
     </row>
     <row r="400" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A400" s="1">
@@ -16710,8 +16818,11 @@
       <c r="D400" s="2" t="s">
         <v>2504</v>
       </c>
-    </row>
-    <row r="401" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+      <c r="E400" s="1" t="s">
+        <v>3080</v>
+      </c>
+    </row>
+    <row r="401" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A401" s="1">
         <v>83</v>
       </c>
@@ -16725,7 +16836,7 @@
         <v>1729</v>
       </c>
     </row>
-    <row r="402" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A402" s="1">
         <v>83</v>
       </c>
@@ -16739,7 +16850,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="403" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A403" s="1">
         <v>84</v>
       </c>
@@ -16753,7 +16864,7 @@
         <v>1609</v>
       </c>
     </row>
-    <row r="404" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A404" s="1">
         <v>84</v>
       </c>
@@ -16767,7 +16878,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="405" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A405" s="1">
         <v>85</v>
       </c>
@@ -16781,7 +16892,7 @@
         <v>2612</v>
       </c>
     </row>
-    <row r="406" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A406" s="1">
         <v>85</v>
       </c>
@@ -16795,7 +16906,7 @@
         <v>1591</v>
       </c>
     </row>
-    <row r="407" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A407" s="1">
         <v>88</v>
       </c>
@@ -16809,7 +16920,7 @@
         <v>2030</v>
       </c>
     </row>
-    <row r="408" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A408" s="1">
         <v>89</v>
       </c>
@@ -16822,8 +16933,11 @@
       <c r="D408" s="2" t="s">
         <v>2527</v>
       </c>
-    </row>
-    <row r="409" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+      <c r="E408" s="1" t="s">
+        <v>3120</v>
+      </c>
+    </row>
+    <row r="409" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A409" s="1">
         <v>89</v>
       </c>
@@ -16836,8 +16950,11 @@
       <c r="D409" s="2" t="s">
         <v>1698</v>
       </c>
-    </row>
-    <row r="410" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+      <c r="E409" s="1" t="s">
+        <v>3120</v>
+      </c>
+    </row>
+    <row r="410" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A410" s="1">
         <v>89</v>
       </c>
@@ -16850,8 +16967,11 @@
       <c r="D410" s="2" t="s">
         <v>1699</v>
       </c>
-    </row>
-    <row r="411" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+      <c r="E410" s="1" t="s">
+        <v>3120</v>
+      </c>
+    </row>
+    <row r="411" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A411" s="1">
         <v>90</v>
       </c>
@@ -16865,7 +16985,7 @@
         <v>980</v>
       </c>
     </row>
-    <row r="412" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A412" s="1">
         <v>90</v>
       </c>
@@ -16879,7 +16999,7 @@
         <v>1716</v>
       </c>
     </row>
-    <row r="413" spans="1:4" ht="80" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:5" ht="80" x14ac:dyDescent="0.25">
       <c r="A413" s="1">
         <v>91</v>
       </c>
@@ -16893,7 +17013,7 @@
         <v>2887</v>
       </c>
     </row>
-    <row r="414" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A414" s="1">
         <v>91</v>
       </c>
@@ -16907,7 +17027,7 @@
         <v>2868</v>
       </c>
     </row>
-    <row r="415" spans="1:4" ht="40" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:5" ht="40" x14ac:dyDescent="0.25">
       <c r="A415" s="1">
         <v>92</v>
       </c>
@@ -16921,7 +17041,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="416" spans="1:4" ht="20" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:5" ht="20" x14ac:dyDescent="0.25">
       <c r="A416" s="1">
         <v>92</v>
       </c>

</xml_diff>